<commit_message>
WIP C4 #540: karta Prodej (UI), stará ukázka smazána, ukázka a šablona v27.10.3, příručky, CHANGELOG, roadmapa, mutace
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018mwHQFWE9rHcnKRUkHnkcJ
</commit_message>
<xml_diff>
--- a/podklady/controlling/SABLONA_PODKLADU_CONTROLLING.xlsx
+++ b/podklady/controlling/SABLONA_PODKLADU_CONTROLLING.xlsx
@@ -594,7 +594,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Šablona pro export předkalkulace struktury verze 3 (list Popis v exportu). Vyrobeno nástrojem nastroje/sablona_podkladu_controlling.py.</t>
+          <t>Šablona pro export předkalkulace struktury verze 4 (list Popis v exportu). Vyrobeno nástrojem nastroje/sablona_podkladu_controlling.py.</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>datum prodeje = podpis SoD / objednané příplatky (dnešní výchozí) / datum odeslání nabídky</t>
+          <t>datum prodeje = tlačítko „Prodáno" v krycím listu (dnešní výchozí) / datum odeslání nabídky</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>ano (dnešní výchozí) / všechny odeslané nabídky</t>
+          <t>všechny (dnešní výchozí) / jen vyhrané (volba exportu)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr"/>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>samostatný řádek bez skupiny / rozpustit do skupin poměrem / jen v souhrnu zakázky</t>
+          <t>jen v souhrnu zakázky, sloupec Zaokrouhlení (dnes) / samostatný řádek bez skupiny / rozpustit do skupin poměrem</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>součet přesně 100 % (zbytek do největší skupiny) / zaokrouhlovat každou zvlášť (dnes)</t>
+          <t>součet přesně 100 % — největší zbytek (dnes) / zaokrouhlovat každou zvlášť</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr"/>

</xml_diff>